<commit_message>
made changes to code
</commit_message>
<xml_diff>
--- a/Extracted_Geographic_Validation.xlsx
+++ b/Extracted_Geographic_Validation.xlsx
@@ -1,20 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\North_American_Management_Work\compare_book_of_negroes_records\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37D10AC2-F68C-42C3-A984-329C4FA27696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="10140" yWindow="0" windowWidth="10455" windowHeight="10905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$51</definedName>
+  </definedNames>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="110">
   <si>
     <t>Notes</t>
   </si>
@@ -25,9 +34,6 @@
     <t>Validation</t>
   </si>
   <si>
-    <t>Coordinates</t>
-  </si>
-  <si>
     <t>City</t>
   </si>
   <si>
@@ -40,6 +46,9 @@
     <t>Country</t>
   </si>
   <si>
+    <t>Final_Coordinates</t>
+  </si>
+  <si>
     <t>George Black, 35, (Lt. Col. Isaac). Freed by Lawrence Hartshorne as certified</t>
   </si>
   <si>
@@ -193,10 +202,7 @@
     <t>-</t>
   </si>
   <si>
-    <t>Sukey</t>
-  </si>
-  <si>
-    <t>Reedy Island, Caroline</t>
+    <t>Caroline</t>
   </si>
   <si>
     <t>Philadelphia</t>
@@ -205,100 +211,103 @@
     <t>little York</t>
   </si>
   <si>
-    <t>New York, Virginia</t>
+    <t>Virginia</t>
   </si>
   <si>
     <t>Madagascar</t>
   </si>
   <si>
-    <t>Virginia</t>
-  </si>
-  <si>
     <t>Jersey</t>
   </si>
   <si>
     <t>Pennsylvania</t>
   </si>
   <si>
-    <t>Woodbury, Charlestown, South Carolina</t>
+    <t>South Carolina</t>
   </si>
   <si>
     <t>Charlestown</t>
   </si>
   <si>
-    <t>Petersburg, Virginia, New York</t>
-  </si>
-  <si>
-    <t>Philadelphia, New York, Dover, Pennsylvania</t>
-  </si>
-  <si>
-    <t>Harrington, New Jersey</t>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>New Jersey</t>
   </si>
   <si>
     <t>Savannah</t>
   </si>
   <si>
-    <t>New Haven, Connecticut</t>
-  </si>
-  <si>
-    <t>Stonington, Connecticut</t>
-  </si>
-  <si>
-    <t>Tappan, New Jersey</t>
-  </si>
-  <si>
-    <t>New Jersey</t>
-  </si>
-  <si>
-    <t>Norfolk, Virginia</t>
-  </si>
-  <si>
-    <t>New Castle County, Pennsylvania</t>
-  </si>
-  <si>
-    <t>Hackensack, New Jersey</t>
-  </si>
-  <si>
-    <t>Isle of White, Virginia</t>
-  </si>
-  <si>
-    <t>Cunningham, Jamaica, West Indies</t>
-  </si>
-  <si>
-    <t>Williamsburgh, Virginia</t>
-  </si>
-  <si>
-    <t>Fredericksburgh, Dutchess County</t>
-  </si>
-  <si>
-    <t>Raritan, New Jersey</t>
+    <t>Connecticut</t>
+  </si>
+  <si>
+    <t>West Indies</t>
+  </si>
+  <si>
+    <t>Dutchess County</t>
   </si>
   <si>
     <t>Antigua</t>
   </si>
   <si>
-    <t>Bergen, New Jersey</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>Yes, Yes</t>
-  </si>
-  <si>
-    <t>Yes, Yes, Yes</t>
-  </si>
-  <si>
-    <t>Yes, Yes, Yes, Yes</t>
-  </si>
-  <si>
-    <t>No, Yes</t>
-  </si>
-  <si>
-    <t>-34.30045, 117.59441</t>
-  </si>
-  <si>
-    <t>39.5145045, -75.5636106, 38.0320305, -77.362363</t>
+    <t>Little York</t>
+  </si>
+  <si>
+    <t>Boston</t>
+  </si>
+  <si>
+    <t>Huruma ward</t>
+  </si>
+  <si>
+    <t>Caroline County</t>
+  </si>
+  <si>
+    <t>Philadelphia County</t>
+  </si>
+  <si>
+    <t>Warren County</t>
+  </si>
+  <si>
+    <t>Jersey County</t>
+  </si>
+  <si>
+    <t>Suffolk County</t>
+  </si>
+  <si>
+    <t>Chatham County</t>
+  </si>
+  <si>
+    <t>Turbo</t>
+  </si>
+  <si>
+    <t>Illinois</t>
+  </si>
+  <si>
+    <t>Massachusetts</t>
+  </si>
+  <si>
+    <t>Georgia</t>
+  </si>
+  <si>
+    <t>Uasin Gishu</t>
+  </si>
+  <si>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>Madagasikara / Madagascar</t>
+  </si>
+  <si>
+    <t>Kenya</t>
+  </si>
+  <si>
+    <t>Antigua and Barbuda</t>
+  </si>
+  <si>
+    <t>38.0320305, -77.362363</t>
   </si>
   <si>
     <t>39.9527237, -75.1635262</t>
@@ -307,293 +316,50 @@
     <t>41.0111483, -90.7462496</t>
   </si>
   <si>
-    <t>40.7127281, -74.0060152, 37.1232245, -78.4927721</t>
+    <t>37.1232245, -78.4927721</t>
   </si>
   <si>
     <t>-18.9249604, 46.4416422</t>
   </si>
   <si>
-    <t>37.1232245, -78.4927721</t>
-  </si>
-  <si>
     <t>39.0848464, -90.3303344</t>
   </si>
   <si>
     <t>40.9699889, -77.7278831</t>
   </si>
   <si>
-    <t>42.3775361, -96.0607187, 42.3778749, -71.0619957, 33.6874388, -80.4363743</t>
-  </si>
-  <si>
-    <t>42.3778749, -71.0619957</t>
-  </si>
-  <si>
-    <t>37.227928, -77.4019268, 37.1232245, -78.4927721, 40.7127281, -74.0060152</t>
-  </si>
-  <si>
-    <t>39.9527237, -75.1635262, 40.7127281, -74.0060152, 51.1251275, 1.3134228, 40.9699889, -77.7278831</t>
-  </si>
-  <si>
-    <t>38.9237244, -75.5777033, 40.0757384, -74.4041622</t>
+    <t>33.6874388, -80.4363743</t>
+  </si>
+  <si>
+    <t>42.3588336, -71.0578303</t>
+  </si>
+  <si>
+    <t>40.7127281, -74.0060152</t>
+  </si>
+  <si>
+    <t>40.0757384, -74.4041622</t>
   </si>
   <si>
     <t>32.0790074, -81.0921335</t>
   </si>
   <si>
-    <t>41.3082138, -72.9250518, 41.6500201, -72.7342163</t>
-  </si>
-  <si>
-    <t>41.3359327, -71.9059042, 41.6500201, -72.7342163</t>
-  </si>
-  <si>
-    <t>41.0248325, -73.9504523, 40.0757384, -74.4041622</t>
-  </si>
-  <si>
-    <t>40.0757384, -74.4041622</t>
-  </si>
-  <si>
-    <t>52.666667, 1.0, 37.1232245, -78.4927721</t>
-  </si>
-  <si>
-    <t>39.6159851, -75.662956, 40.9699889, -77.7278831</t>
-  </si>
-  <si>
-    <t>40.8870781, -74.0410667, 40.0757384, -74.4041622</t>
-  </si>
-  <si>
-    <t>40.7975393, -86.7716793, 37.1232245, -78.4927721</t>
-  </si>
-  <si>
-    <t>37.6439067, -98.4311883, 18.1850507, -77.3947693, 0.5173804, 35.2612102</t>
-  </si>
-  <si>
-    <t>55.8452074, -4.4112604, 37.1232245, -78.4927721</t>
-  </si>
-  <si>
-    <t>-, 41.7194303, -73.7516205</t>
-  </si>
-  <si>
-    <t>40.6958732, -90.8273591, 40.0757384, -74.4041622</t>
+    <t>41.6500201, -72.7342163</t>
+  </si>
+  <si>
+    <t>0.5271707, 35.2451474</t>
+  </si>
+  <si>
+    <t>41.7194303, -73.7516205</t>
   </si>
   <si>
     <t>17.1037152, -61.7904505</t>
-  </si>
-  <si>
-    <t>60.3943055, 5.3259192, 40.0757384, -74.4041622</t>
-  </si>
-  <si>
-    <t>Cranbrook</t>
-  </si>
-  <si>
-    <t>-, -</t>
-  </si>
-  <si>
-    <t>Little York</t>
-  </si>
-  <si>
-    <t>New York, -</t>
-  </si>
-  <si>
-    <t>-, Boston, -</t>
-  </si>
-  <si>
-    <t>Boston</t>
-  </si>
-  <si>
-    <t>Petersburg, -, New York</t>
-  </si>
-  <si>
-    <t>Philadelphia, New York, Dover, -</t>
-  </si>
-  <si>
-    <t>Harrington, -</t>
-  </si>
-  <si>
-    <t>New Haven, -</t>
-  </si>
-  <si>
-    <t>Stonington, -</t>
-  </si>
-  <si>
-    <t>Tappan, -</t>
-  </si>
-  <si>
-    <t>Hackensack, -</t>
-  </si>
-  <si>
-    <t>Cunningham, -, Huruma ward</t>
-  </si>
-  <si>
-    <t>Paisley, -</t>
-  </si>
-  <si>
-    <t>Raritan, -</t>
-  </si>
-  <si>
-    <t>New Castle County, Caroline County</t>
-  </si>
-  <si>
-    <t>Philadelphia County</t>
-  </si>
-  <si>
-    <t>Warren County</t>
-  </si>
-  <si>
-    <t>Jersey County</t>
-  </si>
-  <si>
-    <t>Woodbury County, Suffolk County, -</t>
-  </si>
-  <si>
-    <t>Suffolk County</t>
-  </si>
-  <si>
-    <t>-, -, -</t>
-  </si>
-  <si>
-    <t>Philadelphia County, -, Kent, -</t>
-  </si>
-  <si>
-    <t>Kent County, -</t>
-  </si>
-  <si>
-    <t>Chatham County</t>
-  </si>
-  <si>
-    <t>South Central Connecticut Planning Region, -</t>
-  </si>
-  <si>
-    <t>Southeastern Connecticut Planning Region, -</t>
-  </si>
-  <si>
-    <t>Rockland County, -</t>
-  </si>
-  <si>
-    <t>Norfolk, -</t>
-  </si>
-  <si>
-    <t>New Castle County, -</t>
-  </si>
-  <si>
-    <t>Bergen County, -</t>
-  </si>
-  <si>
-    <t>White County, -</t>
-  </si>
-  <si>
-    <t>Kingman County, -, Turbo</t>
-  </si>
-  <si>
-    <t>Renfrewshire, -</t>
-  </si>
-  <si>
-    <t>-, Dutchess County</t>
-  </si>
-  <si>
-    <t>Henderson County, -</t>
-  </si>
-  <si>
-    <t>Vestland, -</t>
-  </si>
-  <si>
-    <t>Western Australia</t>
-  </si>
-  <si>
-    <t>Delaware, Virginia</t>
-  </si>
-  <si>
-    <t>Illinois</t>
-  </si>
-  <si>
-    <t>Iowa, Massachusetts, South Carolina</t>
-  </si>
-  <si>
-    <t>Massachusetts</t>
-  </si>
-  <si>
-    <t>Virginia, Virginia, New York</t>
-  </si>
-  <si>
-    <t>Pennsylvania, New York, England, Pennsylvania</t>
-  </si>
-  <si>
-    <t>Delaware, New Jersey</t>
-  </si>
-  <si>
-    <t>Georgia</t>
-  </si>
-  <si>
-    <t>Connecticut, Connecticut</t>
-  </si>
-  <si>
-    <t>New York, New Jersey</t>
-  </si>
-  <si>
-    <t>England, Virginia</t>
-  </si>
-  <si>
-    <t>Delaware, Pennsylvania</t>
-  </si>
-  <si>
-    <t>New Jersey, New Jersey</t>
-  </si>
-  <si>
-    <t>Indiana, Virginia</t>
-  </si>
-  <si>
-    <t>Kansas, -, Uasin Gishu</t>
-  </si>
-  <si>
-    <t>Alba / Scotland, Virginia</t>
-  </si>
-  <si>
-    <t>-, New York</t>
-  </si>
-  <si>
-    <t>Illinois, New Jersey</t>
-  </si>
-  <si>
-    <t>-, New Jersey</t>
-  </si>
-  <si>
-    <t>Australia</t>
-  </si>
-  <si>
-    <t>United States, United States</t>
-  </si>
-  <si>
-    <t>United States</t>
-  </si>
-  <si>
-    <t>Madagasikara / Madagascar</t>
-  </si>
-  <si>
-    <t>United States, United States, United States</t>
-  </si>
-  <si>
-    <t>United States, United States, United Kingdom, United States</t>
-  </si>
-  <si>
-    <t>United Kingdom, United States</t>
-  </si>
-  <si>
-    <t>United States, Jamaica, Kenya</t>
-  </si>
-  <si>
-    <t>-, United States</t>
-  </si>
-  <si>
-    <t>Antigua and Barbuda</t>
-  </si>
-  <si>
-    <t>Norge, United States</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -630,13 +396,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -674,7 +448,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -708,6 +482,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -742,9 +517,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -917,11 +693,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H51"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="202.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -947,7 +733,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -973,7 +759,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -999,7 +785,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1025,111 +811,111 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E5" t="s">
-        <v>122</v>
+        <v>58</v>
       </c>
       <c r="F5" t="s">
         <v>58</v>
       </c>
       <c r="G5" t="s">
-        <v>160</v>
+        <v>58</v>
       </c>
       <c r="H5" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" t="s">
+        <v>79</v>
+      </c>
+      <c r="F6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G6" t="s">
+        <v>90</v>
+      </c>
+      <c r="H6" t="s">
         <v>94</v>
       </c>
-      <c r="E6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F6" t="s">
-        <v>138</v>
-      </c>
-      <c r="G6" t="s">
-        <v>161</v>
-      </c>
-      <c r="H6" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E7" t="s">
+        <v>80</v>
+      </c>
+      <c r="F7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G7" t="s">
+        <v>90</v>
+      </c>
+      <c r="H7" t="s">
         <v>95</v>
       </c>
-      <c r="E7" t="s">
-        <v>61</v>
-      </c>
-      <c r="F7" t="s">
-        <v>139</v>
-      </c>
-      <c r="G7" t="s">
-        <v>67</v>
-      </c>
-      <c r="H7" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C8" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D8" t="s">
+        <v>76</v>
+      </c>
+      <c r="E8" t="s">
+        <v>81</v>
+      </c>
+      <c r="F8" t="s">
+        <v>86</v>
+      </c>
+      <c r="G8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H8" t="s">
         <v>96</v>
       </c>
-      <c r="E8" t="s">
-        <v>124</v>
-      </c>
-      <c r="F8" t="s">
-        <v>140</v>
-      </c>
-      <c r="G8" t="s">
-        <v>162</v>
-      </c>
-      <c r="H8" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -1155,137 +941,137 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C10" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E10" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" t="s">
+        <v>90</v>
+      </c>
+      <c r="H10" t="s">
         <v>97</v>
       </c>
-      <c r="E10" t="s">
-        <v>125</v>
-      </c>
-      <c r="F10" t="s">
-        <v>123</v>
-      </c>
-      <c r="G10" t="s">
-        <v>63</v>
-      </c>
-      <c r="H10" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" t="s">
+        <v>91</v>
+      </c>
+      <c r="H11" t="s">
         <v>98</v>
       </c>
-      <c r="E11" t="s">
-        <v>58</v>
-      </c>
-      <c r="F11" t="s">
-        <v>58</v>
-      </c>
-      <c r="G11" t="s">
-        <v>58</v>
-      </c>
-      <c r="H11" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C12" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D12" t="s">
-        <v>99</v>
+        <v>58</v>
       </c>
       <c r="E12" t="s">
         <v>58</v>
       </c>
       <c r="F12" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G12" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="H12" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
       <c r="B13" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C13" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D13" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="E13" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="F13" t="s">
-        <v>141</v>
+        <v>86</v>
       </c>
       <c r="G13" t="s">
-        <v>162</v>
+        <v>90</v>
       </c>
       <c r="H13" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D14" t="s">
-        <v>101</v>
+        <v>58</v>
       </c>
       <c r="E14" t="s">
         <v>58</v>
       </c>
       <c r="F14" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="G14" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="H14" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -1311,7 +1097,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1337,215 +1123,215 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C17" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D17" t="s">
-        <v>99</v>
+        <v>58</v>
       </c>
       <c r="E17" t="s">
         <v>58</v>
       </c>
       <c r="F17" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G17" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="H17" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>24</v>
       </c>
       <c r="B18" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D18" t="s">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="E18" t="s">
-        <v>126</v>
+        <v>58</v>
       </c>
       <c r="F18" t="s">
-        <v>142</v>
+        <v>66</v>
       </c>
       <c r="G18" t="s">
-        <v>163</v>
+        <v>90</v>
       </c>
       <c r="H18" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C19" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D19" t="s">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="E19" t="s">
-        <v>126</v>
+        <v>58</v>
       </c>
       <c r="F19" t="s">
-        <v>142</v>
+        <v>66</v>
       </c>
       <c r="G19" t="s">
-        <v>163</v>
+        <v>90</v>
       </c>
       <c r="H19" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>26</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C20" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D20" t="s">
-        <v>99</v>
+        <v>58</v>
       </c>
       <c r="E20" t="s">
         <v>58</v>
       </c>
       <c r="F20" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G20" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="H20" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>27</v>
       </c>
       <c r="B21" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C21" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D21" t="s">
-        <v>99</v>
+        <v>58</v>
       </c>
       <c r="E21" t="s">
         <v>58</v>
       </c>
       <c r="F21" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G21" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="H21" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C22" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D22" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="E22" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="F22" t="s">
-        <v>141</v>
+        <v>86</v>
       </c>
       <c r="G22" t="s">
-        <v>162</v>
+        <v>90</v>
       </c>
       <c r="H22" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>29</v>
       </c>
       <c r="B23" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C23" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D23" t="s">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="E23" t="s">
-        <v>127</v>
+        <v>83</v>
       </c>
       <c r="F23" t="s">
-        <v>143</v>
+        <v>87</v>
       </c>
       <c r="G23" t="s">
-        <v>164</v>
+        <v>90</v>
       </c>
       <c r="H23" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C24" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D24" t="s">
-        <v>104</v>
+        <v>68</v>
       </c>
       <c r="E24" t="s">
-        <v>128</v>
+        <v>58</v>
       </c>
       <c r="F24" t="s">
-        <v>144</v>
+        <v>68</v>
       </c>
       <c r="G24" t="s">
-        <v>165</v>
+        <v>90</v>
       </c>
       <c r="H24" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -1571,7 +1357,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>32</v>
       </c>
@@ -1597,553 +1383,553 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>33</v>
       </c>
       <c r="B27" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C27" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="D27" t="s">
-        <v>105</v>
+        <v>58</v>
       </c>
       <c r="E27" t="s">
-        <v>129</v>
+        <v>58</v>
       </c>
       <c r="F27" t="s">
-        <v>145</v>
+        <v>65</v>
       </c>
       <c r="G27" t="s">
-        <v>166</v>
+        <v>90</v>
       </c>
       <c r="H27" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>34</v>
       </c>
       <c r="B28" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C28" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D28" t="s">
-        <v>106</v>
+        <v>58</v>
       </c>
       <c r="E28" t="s">
-        <v>130</v>
+        <v>58</v>
       </c>
       <c r="F28" t="s">
-        <v>146</v>
+        <v>69</v>
       </c>
       <c r="G28" t="s">
-        <v>167</v>
+        <v>90</v>
       </c>
       <c r="H28" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C29" t="s">
+        <v>75</v>
+      </c>
+      <c r="D29" t="s">
+        <v>70</v>
+      </c>
+      <c r="E29" t="s">
+        <v>84</v>
+      </c>
+      <c r="F29" t="s">
         <v>88</v>
       </c>
-      <c r="D29" t="s">
-        <v>107</v>
-      </c>
-      <c r="E29" t="s">
-        <v>73</v>
-      </c>
-      <c r="F29" t="s">
-        <v>147</v>
-      </c>
       <c r="G29" t="s">
-        <v>168</v>
+        <v>90</v>
       </c>
       <c r="H29" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>36</v>
       </c>
       <c r="B30" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C30" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D30" t="s">
-        <v>108</v>
+        <v>58</v>
       </c>
       <c r="E30" t="s">
-        <v>131</v>
+        <v>58</v>
       </c>
       <c r="F30" t="s">
-        <v>148</v>
+        <v>71</v>
       </c>
       <c r="G30" t="s">
-        <v>169</v>
+        <v>90</v>
       </c>
       <c r="H30" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>37</v>
       </c>
       <c r="B31" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C31" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D31" t="s">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="E31" t="s">
-        <v>132</v>
+        <v>58</v>
       </c>
       <c r="F31" t="s">
-        <v>149</v>
+        <v>71</v>
       </c>
       <c r="G31" t="s">
-        <v>169</v>
+        <v>90</v>
       </c>
       <c r="H31" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>38</v>
       </c>
       <c r="B32" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C32" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D32" t="s">
-        <v>110</v>
+        <v>58</v>
       </c>
       <c r="E32" t="s">
-        <v>133</v>
+        <v>58</v>
       </c>
       <c r="F32" t="s">
-        <v>150</v>
+        <v>69</v>
       </c>
       <c r="G32" t="s">
-        <v>170</v>
+        <v>90</v>
       </c>
       <c r="H32" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="C33" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D33" t="s">
-        <v>111</v>
+        <v>58</v>
       </c>
       <c r="E33" t="s">
         <v>58</v>
       </c>
       <c r="F33" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="G33" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="H33" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>40</v>
       </c>
       <c r="B34" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="C34" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D34" t="s">
-        <v>112</v>
+        <v>58</v>
       </c>
       <c r="E34" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
       <c r="F34" t="s">
-        <v>151</v>
+        <v>62</v>
       </c>
       <c r="G34" t="s">
-        <v>171</v>
+        <v>90</v>
       </c>
       <c r="H34" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>41</v>
       </c>
       <c r="B35" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C35" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D35" t="s">
-        <v>110</v>
+        <v>58</v>
       </c>
       <c r="E35" t="s">
-        <v>133</v>
+        <v>58</v>
       </c>
       <c r="F35" t="s">
-        <v>150</v>
+        <v>69</v>
       </c>
       <c r="G35" t="s">
-        <v>170</v>
+        <v>90</v>
       </c>
       <c r="H35" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>42</v>
       </c>
       <c r="B36" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C36" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D36" t="s">
-        <v>110</v>
+        <v>58</v>
       </c>
       <c r="E36" t="s">
-        <v>133</v>
+        <v>58</v>
       </c>
       <c r="F36" t="s">
-        <v>150</v>
+        <v>69</v>
       </c>
       <c r="G36" t="s">
-        <v>170</v>
+        <v>90</v>
       </c>
       <c r="H36" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>43</v>
       </c>
       <c r="B37" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C37" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D37" t="s">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="E37" t="s">
-        <v>127</v>
+        <v>83</v>
       </c>
       <c r="F37" t="s">
-        <v>143</v>
+        <v>87</v>
       </c>
       <c r="G37" t="s">
-        <v>164</v>
+        <v>90</v>
       </c>
       <c r="H37" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>44</v>
       </c>
       <c r="B38" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="C38" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D38" t="s">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="E38" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
       <c r="F38" t="s">
-        <v>152</v>
+        <v>65</v>
       </c>
       <c r="G38" t="s">
-        <v>172</v>
+        <v>90</v>
       </c>
       <c r="H38" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>45</v>
       </c>
       <c r="B39" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="C39" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D39" t="s">
-        <v>114</v>
+        <v>58</v>
       </c>
       <c r="E39" t="s">
-        <v>134</v>
+        <v>58</v>
       </c>
       <c r="F39" t="s">
-        <v>153</v>
+        <v>69</v>
       </c>
       <c r="G39" t="s">
-        <v>173</v>
+        <v>90</v>
       </c>
       <c r="H39" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>46</v>
       </c>
       <c r="B40" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C40" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D40" t="s">
-        <v>110</v>
+        <v>58</v>
       </c>
       <c r="E40" t="s">
-        <v>133</v>
+        <v>58</v>
       </c>
       <c r="F40" t="s">
-        <v>150</v>
+        <v>69</v>
       </c>
       <c r="G40" t="s">
-        <v>170</v>
+        <v>90</v>
       </c>
       <c r="H40" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="C41" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D41" t="s">
-        <v>115</v>
+        <v>58</v>
       </c>
       <c r="E41" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
       <c r="F41" t="s">
-        <v>154</v>
+        <v>62</v>
       </c>
       <c r="G41" t="s">
-        <v>174</v>
+        <v>90</v>
       </c>
       <c r="H41" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>48</v>
       </c>
       <c r="B42" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="C42" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D42" t="s">
-        <v>116</v>
+        <v>78</v>
       </c>
       <c r="E42" t="s">
-        <v>135</v>
+        <v>85</v>
       </c>
       <c r="F42" t="s">
-        <v>155</v>
+        <v>89</v>
       </c>
       <c r="G42" t="s">
-        <v>175</v>
+        <v>92</v>
       </c>
       <c r="H42" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>49</v>
       </c>
       <c r="B43" t="s">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="C43" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D43" t="s">
-        <v>117</v>
+        <v>58</v>
       </c>
       <c r="E43" t="s">
-        <v>136</v>
+        <v>58</v>
       </c>
       <c r="F43" t="s">
-        <v>156</v>
+        <v>62</v>
       </c>
       <c r="G43" t="s">
-        <v>176</v>
+        <v>90</v>
       </c>
       <c r="H43" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>50</v>
       </c>
       <c r="B44" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="C44" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="D44" t="s">
-        <v>118</v>
+        <v>58</v>
       </c>
       <c r="E44" t="s">
-        <v>123</v>
+        <v>73</v>
       </c>
       <c r="F44" t="s">
-        <v>157</v>
+        <v>68</v>
       </c>
       <c r="G44" t="s">
-        <v>177</v>
+        <v>90</v>
       </c>
       <c r="H44" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>51</v>
       </c>
       <c r="B45" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="C45" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D45" t="s">
-        <v>112</v>
+        <v>58</v>
       </c>
       <c r="E45" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
       <c r="F45" t="s">
-        <v>151</v>
+        <v>62</v>
       </c>
       <c r="G45" t="s">
-        <v>171</v>
+        <v>90</v>
       </c>
       <c r="H45" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>52</v>
       </c>
       <c r="B46" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="C46" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D46" t="s">
-        <v>119</v>
+        <v>58</v>
       </c>
       <c r="E46" t="s">
-        <v>137</v>
+        <v>58</v>
       </c>
       <c r="F46" t="s">
-        <v>158</v>
+        <v>69</v>
       </c>
       <c r="G46" t="s">
-        <v>178</v>
+        <v>90</v>
       </c>
       <c r="H46" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>53</v>
       </c>
       <c r="B47" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="C47" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D47" t="s">
-        <v>120</v>
+        <v>58</v>
       </c>
       <c r="E47" t="s">
         <v>58</v>
       </c>
       <c r="F47" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="G47" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="H47" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>54</v>
       </c>
@@ -2169,7 +1955,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>55</v>
       </c>
@@ -2195,59 +1981,60 @@
         <v>58</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>56</v>
       </c>
       <c r="B50" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C50" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D50" t="s">
-        <v>110</v>
+        <v>58</v>
       </c>
       <c r="E50" t="s">
-        <v>133</v>
+        <v>58</v>
       </c>
       <c r="F50" t="s">
-        <v>150</v>
+        <v>69</v>
       </c>
       <c r="G50" t="s">
-        <v>170</v>
+        <v>90</v>
       </c>
       <c r="H50" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>57</v>
       </c>
       <c r="B51" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="C51" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D51" t="s">
-        <v>121</v>
+        <v>58</v>
       </c>
       <c r="E51" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
       <c r="F51" t="s">
-        <v>159</v>
+        <v>69</v>
       </c>
       <c r="G51" t="s">
-        <v>179</v>
+        <v>90</v>
       </c>
       <c r="H51" t="s">
-        <v>190</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H51" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
made further changes to the location
</commit_message>
<xml_diff>
--- a/Extracted_Geographic_Validation.xlsx
+++ b/Extracted_Geographic_Validation.xlsx
@@ -1,20 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\North_American_Management_Work\compare_book_of_negroes_records\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B19CDF2C-12A2-4FA6-ABA8-77301C8DB6D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="46230" yWindow="0" windowWidth="25965" windowHeight="10545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$20</definedName>
+  </definedNames>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="98">
   <si>
     <t>Notes</t>
   </si>
@@ -46,215 +55,275 @@
     <t>Final_Coordinates</t>
   </si>
   <si>
-    <t>Richard Lautten, 41, stout make, (James Dowell). Free born in New Castle County, Pennsylvania, at his father's house.</t>
-  </si>
-  <si>
-    <t>Thomas Browne, 40, stout make, 3 long scars each cheek, (George Rapalje). Formerly slave to Ahasmerus Merselis near Hackensack, New Jersey; left him 4 ½ years past by proclamation.</t>
-  </si>
-  <si>
-    <t>William Dunk, 32, stout fellow, (Charles Oliver Bruff). Formerly slave to John Blavalt, Tappan, New Jersey; left him 4½ years past by proclamation.</t>
-  </si>
-  <si>
-    <t>Dick Richards, 22, stout fellow, (William Cassels). Formerly slave to John Wriden, Isle of White, Virginia; left him 4½ years past by proclamation.</t>
-  </si>
-  <si>
-    <t>Joseph, 32, stout fellow, (James Dowell). Formerly slave to Capt. Cunningham, Jamaica, West Indies, who left him free at his death.</t>
-  </si>
-  <si>
-    <t>Isaac, 21, squat stout mulatto, (William Cassels). Formerly slave to John Henderson, Williamsburgh, Virginia; brought off by his parents 5 years ago by proclamation.</t>
-  </si>
-  <si>
-    <t>John Simonsbury, 43, healthy, (Alpheus Palmer). Formerly slave to Charles Collins, Fredericksburgh, Dutchess County; left him four years past by proclamation.</t>
-  </si>
-  <si>
-    <t>Isaac Connor, 49, ailing man, (John Wilson). Formerly slave to Charles Connors, Norfolk, Virginia; left him 4 years past by proclamation.</t>
-  </si>
-  <si>
-    <t>James Perrow, 38, squat little man, (Charles Oliver Bruff). Left free by Alexander Blaes, Raritan landing, New Jersey.</t>
-  </si>
-  <si>
-    <t>Tom Knight, 38, squat little man, (Joseph Inglish). Left Antigua about four years ago. Steven Clarkely.</t>
-  </si>
-  <si>
-    <t>New Castle County, Pennsylvania</t>
-  </si>
-  <si>
-    <t>Hackensack, New Jersey</t>
-  </si>
-  <si>
-    <t>Tappan, New Jersey</t>
-  </si>
-  <si>
-    <t>Isle of White, Virginia</t>
-  </si>
-  <si>
-    <t>Cunningham, Jamaica, West Indies</t>
-  </si>
-  <si>
-    <t>Williamsburgh, Virginia</t>
-  </si>
-  <si>
-    <t>Fredericksburgh, Dutchess County</t>
-  </si>
-  <si>
-    <t>Norfolk, Virginia</t>
-  </si>
-  <si>
-    <t>Raritan, New Jersey</t>
-  </si>
-  <si>
-    <t>Antigua</t>
+    <t>Colin Johnson, 4, M, (Donald Ross).</t>
+  </si>
+  <si>
+    <t>Eisha Johnson, 11, M, (Donald Ross).</t>
+  </si>
+  <si>
+    <t>Patty Johnson, 9 months, M, (Donald Ross).</t>
+  </si>
+  <si>
+    <t>Abraham Thomas, 20, stout lad, B, (Donald Ross). Formerly slave to Lemuel Willet, Fredricksburg, Dutchess County ; says he was born free in the town of West Chester. GBC</t>
+  </si>
+  <si>
+    <t>William Pitt, 32, stout , B, (Robert McQuay). Formerly slave to John Pitt, Nansemond, Virginia; left him &amp; joined the army commanded by General Matthews in the Chesapeak 4 yrs. Past. GBC.</t>
+  </si>
+  <si>
+    <t>Jemima Bull, 26, slender wench, B, (Donald Ross). Formerly slave to Mr. Bull, Rhode Island; left him with the British troops in 1779. GBC</t>
+  </si>
+  <si>
+    <t>Philip bull, 13, fine boy, B, (Donald Ross). Formerly slave to Mr. Bull, Rhode Island; left him with the British troops in 1779.</t>
+  </si>
+  <si>
+    <t>Millia Bull, 6, fine wench, M, (Donald Ross). Formerly slave to Mr. Bull, Rhode Island; left him with the British troops in 1779.</t>
+  </si>
+  <si>
+    <t>Cazar Bull, 1.</t>
+  </si>
+  <si>
+    <t>Isaac Wilson, 22, stout fellow, B, (Hampton Moore). Formerly servant to John Peters near Hamstead, Long Island; says he was born free</t>
+  </si>
+  <si>
+    <t>James Barclett, 59, ordinary fellow, M, (Henry King). Formerly slave to Col. John Washington, Potomack, Virginia; left him about 5 years past. GBC</t>
+  </si>
+  <si>
+    <t>Kate Barclett, 45, ordinary wench, B, (Henry King). Formerly slave to Allen Mozley, Stafford County, Virginia; left him with her husband James Barclett as above. GBC.</t>
+  </si>
+  <si>
+    <t>Nancy Jackson, 11, B, (Alexander McDonald). Formerly servant to Mrs. Maitland, Long Island.</t>
+  </si>
+  <si>
+    <t>Joe Williams, 27, stout fellow, (James Robinson). Formerly servant to Benjamin McVeaugh at Frankfort nigh Philadelphia; left him 6 years past. GBC</t>
+  </si>
+  <si>
+    <t>Billy Knowland, 18, stout fellow, (John Christie). Formerly slave to George Knowland, Nansemond, Virginia; left him 3 yrs. Past. GBC</t>
+  </si>
+  <si>
+    <t>John Williams, 30, stout fellow, (Donald McRimen). Formerly slave to Godolphin Moore nigh Augusta in Georgia; left him 5 years past. GBC</t>
+  </si>
+  <si>
+    <t>Mary, 25, stout squat wench, (Donald McRimen). Formerly slave to Godolphin Moore nigh Augusta in Georgia; left him 5 years past. GBC</t>
+  </si>
+  <si>
+    <t>Samuel Edwards, 36, stout fellow, middle sized, (John Christie). Says he is free and lived as a hired servant with Mr. Dickenson of Philadelphia.</t>
+  </si>
+  <si>
+    <t>Betsey Fountain, 21, stout wench, (John Cowling). Formerly slave to William Hascomb of Northumberland County, Virginia; left him 7 years past. GBC</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Fredricksburg, Dutchess County, West Chester</t>
+  </si>
+  <si>
+    <t>Nansemond, Virginia, Chesapeak</t>
+  </si>
+  <si>
+    <t>Rhode Island</t>
+  </si>
+  <si>
+    <t>Hamstead, Long Island</t>
+  </si>
+  <si>
+    <t>Potomack, Virginia</t>
+  </si>
+  <si>
+    <t>Stafford County, Virginia</t>
+  </si>
+  <si>
+    <t>Long Island</t>
+  </si>
+  <si>
+    <t>Frankfort, Philadelphia</t>
+  </si>
+  <si>
+    <t>Nansemond, Virginia</t>
+  </si>
+  <si>
+    <t>Augusta, Georgia</t>
+  </si>
+  <si>
+    <t>Philadelphia</t>
+  </si>
+  <si>
+    <t>Northumberland County, Virginia</t>
+  </si>
+  <si>
+    <t>Yes, Yes, Yes</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
   <si>
     <t>Yes, Yes</t>
   </si>
   <si>
-    <t>Yes, Yes, Yes</t>
-  </si>
-  <si>
-    <t>No, Yes</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Hackensack</t>
-  </si>
-  <si>
-    <t>Tappan</t>
-  </si>
-  <si>
-    <t>Cunningham</t>
-  </si>
-  <si>
-    <t>Williamsburgh</t>
-  </si>
-  <si>
-    <t>Raritan</t>
-  </si>
-  <si>
-    <t>Isle of White</t>
-  </si>
-  <si>
-    <t>New Castle County</t>
-  </si>
-  <si>
-    <t>Bergen County</t>
-  </si>
-  <si>
-    <t>Rockland County</t>
-  </si>
-  <si>
-    <t>White County</t>
-  </si>
-  <si>
-    <t>Kingman County</t>
-  </si>
-  <si>
-    <t>Renfrewshire</t>
-  </si>
-  <si>
-    <t>Dutchess County</t>
-  </si>
-  <si>
-    <t>Norfolk</t>
-  </si>
-  <si>
-    <t>Henderson County</t>
+    <t>Aurora, West Chester</t>
+  </si>
+  <si>
+    <t>Suffolk</t>
+  </si>
+  <si>
+    <t>Raleigh</t>
+  </si>
+  <si>
+    <t>Bolivar</t>
+  </si>
+  <si>
+    <t>Augusta</t>
+  </si>
+  <si>
+    <t>Fredricksburg</t>
+  </si>
+  <si>
+    <t>Nansemond, Chesapeak</t>
+  </si>
+  <si>
+    <t>Potomack</t>
+  </si>
+  <si>
+    <t>Nansemond</t>
+  </si>
+  <si>
+    <t>Kendall County, Dutchess County, Chester County</t>
+  </si>
+  <si>
+    <t>Caroline County</t>
+  </si>
+  <si>
+    <t>Wake County</t>
+  </si>
+  <si>
+    <t>Jefferson County</t>
+  </si>
+  <si>
+    <t>Stafford County</t>
+  </si>
+  <si>
+    <t>Franklin County, Philadelphia County</t>
+  </si>
+  <si>
+    <t>Richmond County</t>
+  </si>
+  <si>
+    <t>Philadelphia County</t>
+  </si>
+  <si>
+    <t>Northumberland County</t>
+  </si>
+  <si>
+    <t>Illinois, New York, Pennsylvania</t>
+  </si>
+  <si>
+    <t>Virginia, Maryland</t>
+  </si>
+  <si>
+    <t>North Carolina, New York</t>
+  </si>
+  <si>
+    <t>West Virginia, Virginia</t>
+  </si>
+  <si>
+    <t>Virginia</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>Kentucky, Pennsylvania</t>
+  </si>
+  <si>
+    <t>Georgia</t>
   </si>
   <si>
     <t>Pennsylvania</t>
   </si>
   <si>
-    <t>New Jersey</t>
-  </si>
-  <si>
-    <t>Virginia</t>
-  </si>
-  <si>
-    <t>Kansas</t>
-  </si>
-  <si>
-    <t>New York</t>
+    <t>Pennsylvania, Virginia</t>
   </si>
   <si>
     <t>United States</t>
   </si>
   <si>
-    <t>Jamaica</t>
-  </si>
-  <si>
-    <t>Antigua and Barbuda</t>
-  </si>
-  <si>
-    <t>New Castle County, Pennsylvania, United States - New Castle County - Pennsylvania - United States</t>
-  </si>
-  <si>
-    <t>Hackensack, Bergen County, New Jersey, United States - Hackensack, New Jersey - Hackensack, United States - Hackensack - Bergen County - New Jersey - United States</t>
-  </si>
-  <si>
-    <t>Tappan, Tappan, Rockland County, New Jersey, United States - Tappan, New Jersey - Tappan, United States - Tappan - Rockland County - New Jersey - United States</t>
-  </si>
-  <si>
-    <t>Isle of White - White County - Virginia - United States</t>
-  </si>
-  <si>
-    <t>Cunningham, Kansas - Cunningham, Jamaica - Cunningham - Kingman County - Kansas - Jamaica</t>
-  </si>
-  <si>
-    <t>Williamsburgh, United States - Williamsburgh - Renfrewshire - Virginia - United States</t>
-  </si>
-  <si>
-    <t>Dutchess County, New York, United States - Dutchess County - New York - United States</t>
-  </si>
-  <si>
-    <t>Norfolk, Virginia, United States - Norfolk - Virginia - United States</t>
-  </si>
-  <si>
-    <t>Raritan, New Jersey - Raritan, United States - Raritan - Henderson County - New Jersey - United States</t>
-  </si>
-  <si>
-    <t>Antigua, Antigua and Barbuda - Antigua - Antigua and Barbuda</t>
-  </si>
-  <si>
-    <t>40.9947347, -80.3191623 - 39.6159851, -75.662956 - 40.9699889, -77.7278831 - 39.7837304, -100.445882</t>
-  </si>
-  <si>
-    <t>40.8870781, -74.0410667 - 40.8870781, -74.0410667 - 40.8870781, -74.0410667 - 40.8870781, -74.0410667 - 40.9678345, -74.0563254 - 40.0757384, -74.4041622 - 39.7837304, -100.445882</t>
-  </si>
-  <si>
-    <t>41.0225692, -73.9569505 - 41.0106971, -73.9911073 - 41.0248325, -73.9504523 - 41.0248325, -73.9504523 - 41.1519319, -74.0357266 - 40.0757384, -74.4041622 - 39.7837304, -100.445882</t>
-  </si>
-  <si>
-    <t>40.7975393, -86.7716793 - 38.0632329, -88.1577725 - 37.1232245, -78.4927721 - 39.7837304, -100.445882</t>
-  </si>
-  <si>
-    <t>37.6439067, -98.4311883 - 18.0043137, -76.7734388 - 37.6439067, -98.4311883 - 37.5420937, -98.122172 - 38.27312, -98.5821872 - 18.1850507, -77.3947693</t>
-  </si>
-  <si>
-    <t>40.8013344, -111.9410495 - 55.8452074, -4.4112604 - 55.833333, -4.5 - 37.1232245, -78.4927721 - 39.7837304, -100.445882</t>
-  </si>
-  <si>
-    <t>41.7194303, -73.7516205 - 41.7194303, -73.7516205 - 40.7127281, -74.0060152 - 39.7837304, -100.445882</t>
-  </si>
-  <si>
-    <t>36.8493695, -76.2899539 - 52.666667, 1.0 - 37.1232245, -78.4927721 - 39.7837304, -100.445882</t>
-  </si>
-  <si>
-    <t>40.567181, -74.634683 - 40.6958732, -90.8273591 - 40.6958732, -90.8273591 - 32.182598, -95.7893178 - 40.0757384, -74.4041622 - 39.7837304, -100.445882</t>
-  </si>
-  <si>
-    <t>17.1037152, -61.7904505 - 17.1037152, -61.7904505 - 17.2234721, -61.9554608</t>
+    <t>41.7107066, -88.2692377 -- 41.7107066, -88.2692377 -- 41.7571701, -88.3147539 -- 41.7571701, -88.3147539 -- 39.9597389, -75.6044609 -- 39.9597389, -75.6044609 -- 29.943885, -98.7258845 -- 29.943885, -98.7258845 -- 41.7194303, -73.7516205 -- 41.7194303, -73.7516205 -- 39.9829308, -75.7652424 -- 39.9829308, -75.7652424 -- 40.0796606, -89.4337288 -- 40.0796606, -89.4337288 -- 40.7127281, -74.0060152 -- 40.7127281, -74.0060152 -- 40.9699889, -77.7278831 -- 40.9699889, -77.7278831 -- 39.7837304, -100.445882 -- 39.7837304, -100.445882</t>
+  </si>
+  <si>
+    <t>36.7670938, -76.5307823 -- 36.7670938, -76.5307823 -- 38.8000953, -75.7418774 -- 38.8000953, -75.7418774 -- 40.8832318, -72.8578027 -- 40.8832318, -72.8578027 -- 38.0320305, -77.362363 -- 38.0320305, -77.362363 -- 37.1232245, -78.4927721 -- 37.1232245, -78.4927721 -- 39.5162401, -76.9382069 -- 39.5162401, -76.9382069 -- 39.7837304, -100.445882 -- 39.7837304, -100.445882</t>
+  </si>
+  <si>
+    <t>41.7962409, -71.5992372 -- 41.7962409, -71.5992372 -- 39.7837304, -100.445882 -- 39.7837304, -100.445882</t>
+  </si>
+  <si>
+    <t>35.8544627, -78.7097905 -- 35.8544627, -78.7097905 -- 40.8514971, -73.0994297 -- 40.8514971, -73.0994297 -- 35.7803977, -78.6390989 -- 35.7803977, -78.6390989 -- 35.7979355, -78.6118311 -- 35.7979355, -78.6118311 -- 35.6729639, -79.0392919 -- 35.6729639, -79.0392919 -- 40.7127281, -74.0060152 -- 40.7127281, -74.0060152 -- 39.7837304, -100.445882 -- 39.7837304, -100.445882</t>
+  </si>
+  <si>
+    <t>39.3179629, -77.7496548 -- 39.3179629, -77.7496548 -- 39.3179629, -77.7496548 -- 33.7702263, -90.8519798 -- 33.7702263, -90.8519798 -- 29.834772, -94.1704496 -- 29.834772, -94.1704496 -- 38.4758406, -80.8408415 -- 38.4758406, -80.8408415 -- 37.1232245, -78.4927721 -- 37.1232245, -78.4927721 -- 39.7837304, -100.445882 -- 39.7837304, -100.445882</t>
+  </si>
+  <si>
+    <t>38.4167265, -77.4579783 -- 38.4167265, -77.4579783 -- 38.4167265, -77.4579783 -- 37.1232245, -78.4927721 -- 37.1232245, -78.4927721 -- 39.7837304, -100.445882 -- 39.7837304, -100.445882</t>
+  </si>
+  <si>
+    <t>40.8514971, -73.0994297 -- 40.8514971, -73.0994297 -- 40.8514971, -73.0994297 -- 40.7127281, -74.0060152 -- 40.7127281, -74.0060152 -- 39.7837304, -100.445882 -- 39.7837304, -100.445882</t>
+  </si>
+  <si>
+    <t>38.2009055, -84.8732836 -- 38.2009055, -84.8732836 -- 39.9527237, -75.1635262 -- 39.9527237, -75.1635262 -- 33.2002659, -95.2231752 -- 33.2002659, -95.2231752 -- 40.0114538, -75.1326504 -- 40.0114538, -75.1326504 -- 37.5726028, -85.1551411 -- 37.5726028, -85.1551411 -- 40.9699889, -77.7278831 -- 40.9699889, -77.7278831 -- 39.7837304, -100.445882 -- 39.7837304, -100.445882</t>
+  </si>
+  <si>
+    <t>36.7670938, -76.5307823 -- 36.7670938, -76.5307823 -- 36.7670938, -76.5307823 -- 40.8832318, -72.8578027 -- 40.8832318, -72.8578027 -- 37.1232245, -78.4927721 -- 37.1232245, -78.4927721 -- 39.7837304, -100.445882 -- 39.7837304, -100.445882</t>
+  </si>
+  <si>
+    <t>33.4709714, -81.9748429 -- 33.4709714, -81.9748429 -- 33.4709714, -81.9748429 -- 40.5834557, -74.1496048 -- 40.5834557, -74.1496048 -- 32.3293809, -83.1137366 -- 32.3293809, -83.1137366 -- 39.7837304, -100.445882 -- 39.7837304, -100.445882</t>
+  </si>
+  <si>
+    <t>39.9527237, -75.1635262 -- 39.9527237, -75.1635262 -- 39.9527237, -75.1635262 -- 40.0114538, -75.1326504 -- 40.0114538, -75.1326504 -- 40.9699889, -77.7278831 -- 40.9699889, -77.7278831 -- 39.7837304, -100.445882 -- 39.7837304, -100.445882</t>
+  </si>
+  <si>
+    <t>40.8488473, -76.6943741 -- 40.8488473, -76.6943741 -- 40.9699889, -77.7278831 -- 40.9699889, -77.7278831 -- 37.1232245, -78.4927721 -- 37.1232245, -78.4927721 -- 39.7837304, -100.445882 -- 39.7837304, -100.445882</t>
+  </si>
+  <si>
+    <t>Fredricksburg -- Fredricksburg, United States -- Aurora -- Aurora, United States -- West Chester -- West Chester, United States -- Kendall County -- Kendall County, United States -- Dutchess County -- Dutchess County, United States -- Chester County -- Chester County, United States -- Illinois -- Illinois, United States -- New York -- New York, United States -- Pennsylvania -- Pennsylvania, United States -- United States -- United States, United States</t>
+  </si>
+  <si>
+    <t>Nansemond -- Nansemond, United States -- Chesapeak -- Chesapeak, United States -- Suffolk -- Suffolk, United States -- Caroline County -- Caroline County, United States -- Virginia -- Virginia, United States -- Maryland -- Maryland, United States -- United States -- United States, United States</t>
+  </si>
+  <si>
+    <t>Rhode Island, United States -- Rhode Island -- United States -- United States, United States</t>
+  </si>
+  <si>
+    <t>Hamstead -- Hamstead, United States -- Long Island -- Long Island, United States -- Raleigh -- Raleigh, United States -- Wake County -- Wake County, United States -- North Carolina -- North Carolina, United States -- New York -- New York, United States -- United States -- United States, United States</t>
+  </si>
+  <si>
+    <t>Potomack, Bolivar, Jefferson County, West Virginia, Virginia, United States -- Potomack -- Potomack, United States -- Bolivar -- Bolivar, United States -- Jefferson County -- Jefferson County, United States -- West Virginia -- West Virginia, United States -- Virginia -- Virginia, United States -- United States -- United States, United States</t>
+  </si>
+  <si>
+    <t>Stafford County, Virginia, United States -- Stafford County -- Stafford County, United States -- Virginia -- Virginia, United States -- United States -- United States, United States</t>
+  </si>
+  <si>
+    <t>Long Island, New York, United States -- Long Island -- Long Island, United States -- New York -- New York, United States -- United States -- United States, United States</t>
+  </si>
+  <si>
+    <t>Frankfort -- Frankfort, United States -- Philadelphia -- Philadelphia, United States -- Franklin County -- Franklin County, United States -- Philadelphia County -- Philadelphia County, United States -- Kentucky -- Kentucky, United States -- Pennsylvania -- Pennsylvania, United States -- United States -- United States, United States</t>
+  </si>
+  <si>
+    <t>Nansemond, Suffolk, Virginia, United States -- Nansemond -- Nansemond, United States -- Suffolk -- Suffolk, United States -- Virginia -- Virginia, United States -- United States -- United States, United States</t>
+  </si>
+  <si>
+    <t>Augusta, Richmond County, Georgia, United States -- Augusta -- Augusta, United States -- Richmond County -- Richmond County, United States -- Georgia -- Georgia, United States -- United States -- United States, United States</t>
+  </si>
+  <si>
+    <t>Philadelphia, Philadelphia County, Pennsylvania, United States -- Philadelphia -- Philadelphia, United States -- Philadelphia County -- Philadelphia County, United States -- Pennsylvania -- Pennsylvania, United States -- United States -- United States, United States</t>
+  </si>
+  <si>
+    <t>Northumberland County -- Northumberland County, United States -- Pennsylvania -- Pennsylvania, United States -- Virginia -- Virginia, United States -- United States -- United States, United States</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -291,13 +360,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -335,7 +412,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -369,6 +446,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -403,9 +481,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -578,11 +657,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="173" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="45.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="255.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -614,327 +704,616 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="G2" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="H2" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="I2" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="J2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F3" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G3" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="H3" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="I3" t="s">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="J3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="G4" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="H4" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="I4" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="J4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F5" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="G5" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="H5" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="I5" t="s">
-        <v>61</v>
+        <v>86</v>
       </c>
       <c r="J5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="F6" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G6" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="H6" t="s">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="I6" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="J6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="G7" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="H7" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="I7" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="J7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" t="s">
         <v>32</v>
       </c>
-      <c r="D8" t="s">
-        <v>34</v>
-      </c>
-      <c r="E8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F8" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" t="s">
-        <v>54</v>
-      </c>
       <c r="H8" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="I8" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="J8" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F9" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="G9" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="H9" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="I9" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="J9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="E10" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="G10" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="H10" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="I10" t="s">
-        <v>66</v>
+        <v>29</v>
       </c>
       <c r="J10" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" t="s">
         <v>33</v>
       </c>
-      <c r="D11" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" t="s">
-        <v>34</v>
-      </c>
       <c r="F11" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="G11" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="H11" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="I11" t="s">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="J11" t="s">
         <v>77</v>
       </c>
     </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E12" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" t="s">
+        <v>57</v>
+      </c>
+      <c r="G12" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12" t="s">
+        <v>73</v>
+      </c>
+      <c r="I12" t="s">
+        <v>90</v>
+      </c>
+      <c r="J12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G13" t="s">
+        <v>67</v>
+      </c>
+      <c r="H13" t="s">
+        <v>73</v>
+      </c>
+      <c r="I13" t="s">
+        <v>91</v>
+      </c>
+      <c r="J13" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" t="s">
+        <v>36</v>
+      </c>
+      <c r="F14" t="s">
+        <v>29</v>
+      </c>
+      <c r="G14" t="s">
+        <v>68</v>
+      </c>
+      <c r="H14" t="s">
+        <v>73</v>
+      </c>
+      <c r="I14" t="s">
+        <v>92</v>
+      </c>
+      <c r="J14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" t="s">
+        <v>59</v>
+      </c>
+      <c r="G15" t="s">
+        <v>69</v>
+      </c>
+      <c r="H15" t="s">
+        <v>73</v>
+      </c>
+      <c r="I15" t="s">
+        <v>93</v>
+      </c>
+      <c r="J15" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" t="s">
+        <v>53</v>
+      </c>
+      <c r="F16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G16" t="s">
+        <v>67</v>
+      </c>
+      <c r="H16" t="s">
+        <v>73</v>
+      </c>
+      <c r="I16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J16" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" t="s">
+        <v>49</v>
+      </c>
+      <c r="E17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" t="s">
+        <v>60</v>
+      </c>
+      <c r="G17" t="s">
+        <v>70</v>
+      </c>
+      <c r="H17" t="s">
+        <v>73</v>
+      </c>
+      <c r="I17" t="s">
+        <v>95</v>
+      </c>
+      <c r="J17" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" t="s">
+        <v>49</v>
+      </c>
+      <c r="E18" t="s">
+        <v>29</v>
+      </c>
+      <c r="F18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" t="s">
+        <v>70</v>
+      </c>
+      <c r="H18" t="s">
+        <v>73</v>
+      </c>
+      <c r="I18" t="s">
+        <v>95</v>
+      </c>
+      <c r="J18" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" t="s">
+        <v>29</v>
+      </c>
+      <c r="F19" t="s">
+        <v>61</v>
+      </c>
+      <c r="G19" t="s">
+        <v>71</v>
+      </c>
+      <c r="H19" t="s">
+        <v>73</v>
+      </c>
+      <c r="I19" t="s">
+        <v>96</v>
+      </c>
+      <c r="J19" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" t="s">
+        <v>29</v>
+      </c>
+      <c r="E20" t="s">
+        <v>29</v>
+      </c>
+      <c r="F20" t="s">
+        <v>62</v>
+      </c>
+      <c r="G20" t="s">
+        <v>72</v>
+      </c>
+      <c r="H20" t="s">
+        <v>73</v>
+      </c>
+      <c r="I20" t="s">
+        <v>97</v>
+      </c>
+      <c r="J20" t="s">
+        <v>85</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:J20" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>